<commit_message>
Add EV/sales-to-growth + negative-EV deep-value archetypes
arch_exceptional_evsg (1,623): a fast grower priced at an EXCEPTIONALLY
low EV/sales relative to that growth (EVSG = EV/sales ÷ revenue-growth%,
the capital-structure-neutral analog of PSG). No organic-vs-total revenue
split exists, so total revenue growth proxies organic. Lower bounds on
ev_sales (>=0.15) and evsg drop razor-margin traders / near-zero-EV
artifacts; light quality gate excludes pre-revenue burn shells. New
`evsg` column in derive.

arch_negative_ev_value (6,217): market cap at/below net cash (negative or
tiny EV — paid to own the operating business) OR price well below book,
with a survivability gate (positive cash flow OR big net-cash cushion) so
the cash is protective, not melting-ice (the Belluscura lesson). 920
negative-EV names + deep sub-book.

Universe now 58 archetypes; all 10 books regenerated, 0 nan/inf.
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -56493,10 +56493,8 @@
           <t>EV / EBIT</t>
         </is>
       </c>
-      <c r="C30" s="37" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="C30" s="24" t="n">
+        <v>-0.6718202981877625</v>
       </c>
       <c r="D30" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Mid-drive merge #5 (union A+B, ~85%) + regenerate all 11 books
Union of the dual enrichers folded in (22,727 names, 85%). asleep_at_wheel
901->1685, templeton_pessimism 2356->2965. Includes the new country x archetype
inflection book. All 11 books regenerated; 0 nan/inf verified.
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -55021,42 +55021,42 @@
       </c>
       <c r="C27" s="26" t="inlineStr">
         <is>
-          <t>NBA.LS</t>
+          <t>R4.MC</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
         <is>
-          <t>Novabase S.G.P.S., S.A.</t>
+          <t>Renta 4 Banco, S.A.</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>PT</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G27" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="H27" s="22" t="n">
-        <v>306669280</v>
-      </c>
-      <c r="I27" s="23" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+        <v>777240192</v>
+      </c>
+      <c r="I27" s="25" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="J27" s="24" t="n">
-        <v>0.3964734355710773</v>
+        <v>0.3984065238614438</v>
       </c>
       <c r="K27" s="24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="17" customHeight="1">
@@ -55065,22 +55065,22 @@
       </c>
       <c r="C28" s="26" t="inlineStr">
         <is>
-          <t>EYAPS.AT</t>
+          <t>NBA.LS</t>
         </is>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Thessaloniki Water Supply &amp; Sewerage Co S.A.</t>
+          <t>Novabase S.G.P.S., S.A.</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>GR</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
@@ -55089,18 +55089,18 @@
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>164257504</v>
-      </c>
-      <c r="I28" s="25" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+        <v>306669280</v>
+      </c>
+      <c r="I28" s="23" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="J28" s="24" t="n">
-        <v>0.3944587233284998</v>
+        <v>0.3964734355710773</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-render all 16 books on fixed gates, rankings, and OTC partition
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -31463,12 +31463,12 @@
       </c>
       <c r="C17" s="26" t="inlineStr">
         <is>
-          <t>INAB</t>
+          <t>JFU</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>IN8bio Inc. Common Stock</t>
+          <t>9F Inc.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -31478,16 +31478,16 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>13041940</v>
+        <v>30610668</v>
       </c>
       <c r="I17" s="25" t="inlineStr">
         <is>
@@ -31495,18 +31495,16 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.7705145530704575</v>
+        <v>0.7698883687256359</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>1</v>
+        <v>0.714</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>0.587981</v>
-      </c>
-      <c r="M17" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.055835366</v>
+      </c>
+      <c r="M17" s="24" t="n">
+        <v>0.10559772</v>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
@@ -31515,12 +31513,12 @@
       </c>
       <c r="C18" s="26" t="inlineStr">
         <is>
-          <t>JFU</t>
+          <t>SF-PB</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>9F Inc.</t>
+          <t>Stifel Financial Corp.</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -31530,16 +31528,16 @@
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>30610668</v>
+        <v>1712339787.48</v>
       </c>
       <c r="I18" s="25" t="inlineStr">
         <is>
@@ -31547,16 +31545,16 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.7698883687256359</v>
+        <v>0.7680252075321161</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.714</v>
+        <v>0.667</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.055835366</v>
+        <v>0.6591588</v>
       </c>
       <c r="M18" s="24" t="n">
-        <v>0.10559772</v>
+        <v>0.3010436842474461</v>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
@@ -31565,12 +31563,12 @@
       </c>
       <c r="C19" s="26" t="inlineStr">
         <is>
-          <t>SF-PB</t>
+          <t>TIGR</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Stifel Financial Corp.</t>
+          <t>Up Fintech Holding Limited</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -31589,7 +31587,7 @@
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>1712339787.48</v>
+        <v>838106112</v>
       </c>
       <c r="I19" s="25" t="inlineStr">
         <is>
@@ -31597,16 +31595,16 @@
         </is>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.7680252075321161</v>
+        <v>0.7574812361405707</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>0.6591588</v>
+        <v>0.9904963</v>
       </c>
       <c r="M19" s="24" t="n">
-        <v>0.3010436842474461</v>
+        <v>1.4758615</v>
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
@@ -31615,12 +31613,12 @@
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
-          <t>TIGR</t>
+          <t>XNET</t>
         </is>
       </c>
       <c r="D20" s="18" t="inlineStr">
         <is>
-          <t>Up Fintech Holding Limited</t>
+          <t>Xunlei Ltd</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -31630,7 +31628,7 @@
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
@@ -31639,7 +31637,7 @@
         </is>
       </c>
       <c r="H20" s="22" t="n">
-        <v>838106112</v>
+        <v>341184288</v>
       </c>
       <c r="I20" s="25" t="inlineStr">
         <is>
@@ -31647,16 +31645,16 @@
         </is>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.7574812361405707</v>
+        <v>0.7557172277310804</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>1</v>
+        <v>0.778</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>0.9904963</v>
+        <v>0.24528648</v>
       </c>
       <c r="M20" s="24" t="n">
-        <v>1.4758615</v>
+        <v>0.6895314</v>
       </c>
     </row>
     <row r="21" ht="17" customHeight="1">
@@ -31665,12 +31663,12 @@
       </c>
       <c r="C21" s="26" t="inlineStr">
         <is>
-          <t>XNET</t>
+          <t>080010.KQ</t>
         </is>
       </c>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Xunlei Ltd</t>
+          <t>eSang Networks Co.,Ltd</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
@@ -31680,16 +31678,16 @@
       </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G21" s="21" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H21" s="22" t="n">
-        <v>341184288</v>
+        <v>40157934.09804344</v>
       </c>
       <c r="I21" s="25" t="inlineStr">
         <is>
@@ -31697,16 +31695,16 @@
         </is>
       </c>
       <c r="J21" s="24" t="n">
-        <v>0.7557172277310804</v>
+        <v>0.7539593481207859</v>
       </c>
       <c r="K21" s="24" t="n">
-        <v>0.778</v>
+        <v>1</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>0.24528648</v>
+        <v>0.4318499805098363</v>
       </c>
       <c r="M21" s="24" t="n">
-        <v>0.6895314</v>
+        <v>0.5690626668871859</v>
       </c>
     </row>
     <row r="22" ht="17" customHeight="1">
@@ -31715,12 +31713,12 @@
       </c>
       <c r="C22" s="26" t="inlineStr">
         <is>
-          <t>080010.KQ</t>
+          <t>SSBI</t>
         </is>
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>eSang Networks Co.,Ltd</t>
+          <t>Summit State Bank</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
@@ -31739,7 +31737,7 @@
         </is>
       </c>
       <c r="H22" s="22" t="n">
-        <v>40157934.09804344</v>
+        <v>91686464</v>
       </c>
       <c r="I22" s="25" t="inlineStr">
         <is>
@@ -31747,16 +31745,16 @@
         </is>
       </c>
       <c r="J22" s="24" t="n">
-        <v>0.7539593481207859</v>
+        <v>0.7379038867123762</v>
       </c>
       <c r="K22" s="24" t="n">
         <v>1</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>0.4318499805098363</v>
+        <v>0.8930992684661166</v>
       </c>
       <c r="M22" s="24" t="n">
-        <v>0.5690626668871859</v>
+        <v>2.52503274489824</v>
       </c>
     </row>
     <row r="23" ht="17" customHeight="1">
@@ -31765,17 +31763,17 @@
       </c>
       <c r="C23" s="26" t="inlineStr">
         <is>
-          <t>SSBI</t>
+          <t>ELC.V</t>
         </is>
       </c>
       <c r="D23" s="18" t="inlineStr">
         <is>
-          <t>Summit State Bank</t>
+          <t>Elysee Development Corp.</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F23" s="20" t="inlineStr">
@@ -31785,11 +31783,11 @@
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H23" s="22" t="n">
-        <v>91686464</v>
+        <v>13155677.1619345</v>
       </c>
       <c r="I23" s="25" t="inlineStr">
         <is>
@@ -31797,16 +31795,16 @@
         </is>
       </c>
       <c r="J23" s="24" t="n">
-        <v>0.7379038867123762</v>
+        <v>0.7363425284206518</v>
       </c>
       <c r="K23" s="24" t="n">
         <v>1</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>0.8930992684661166</v>
+        <v>0.8050134601820504</v>
       </c>
       <c r="M23" s="24" t="n">
-        <v>2.52503274489824</v>
+        <v>2.949994818357315</v>
       </c>
     </row>
     <row r="24" ht="17" customHeight="1">
@@ -31815,31 +31813,31 @@
       </c>
       <c r="C24" s="26" t="inlineStr">
         <is>
-          <t>ELC.V</t>
+          <t>IMPP</t>
         </is>
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>Elysee Development Corp.</t>
+          <t>Imperial Petroleum Inc./Marshall Islands</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="G24" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H24" s="22" t="n">
-        <v>13155677.1619345</v>
+        <v>219738368</v>
       </c>
       <c r="I24" s="25" t="inlineStr">
         <is>
@@ -31847,16 +31845,16 @@
         </is>
       </c>
       <c r="J24" s="24" t="n">
-        <v>0.7363425284206518</v>
+        <v>0.7361943217674636</v>
       </c>
       <c r="K24" s="24" t="n">
-        <v>1</v>
+        <v>0.857</v>
       </c>
       <c r="L24" s="24" t="n">
-        <v>0.8050134601820504</v>
+        <v>0.39409667</v>
       </c>
       <c r="M24" s="24" t="n">
-        <v>2.949994818357315</v>
+        <v>1.1527194</v>
       </c>
     </row>
     <row r="25" ht="17" customHeight="1">
@@ -31865,12 +31863,12 @@
       </c>
       <c r="C25" s="26" t="inlineStr">
         <is>
-          <t>IMPP</t>
+          <t>CRON</t>
         </is>
       </c>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Imperial Petroleum Inc./Marshall Islands</t>
+          <t>Cronos Group Inc.</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -31880,16 +31878,16 @@
       </c>
       <c r="F25" s="20" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G25" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="H25" s="22" t="n">
-        <v>219738368</v>
+        <v>1049990336</v>
       </c>
       <c r="I25" s="25" t="inlineStr">
         <is>
@@ -31897,16 +31895,16 @@
         </is>
       </c>
       <c r="J25" s="24" t="n">
-        <v>0.7361943217674636</v>
+        <v>0.7342596256130441</v>
       </c>
       <c r="K25" s="24" t="n">
-        <v>0.857</v>
+        <v>0.875</v>
       </c>
       <c r="L25" s="24" t="n">
-        <v>0.39409667</v>
+        <v>0.98458296</v>
       </c>
       <c r="M25" s="24" t="n">
-        <v>1.1527194</v>
+        <v>6.581567</v>
       </c>
     </row>
     <row r="26" ht="17" customHeight="1">
@@ -31915,12 +31913,12 @@
       </c>
       <c r="C26" s="26" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>KPLT</t>
         </is>
       </c>
       <c r="D26" s="18" t="inlineStr">
         <is>
-          <t>Cronos Group Inc.</t>
+          <t>Katapult Holdings Inc. Common Stock</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
@@ -31930,16 +31928,16 @@
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H26" s="22" t="n">
-        <v>1049990336</v>
+        <v>32688298</v>
       </c>
       <c r="I26" s="25" t="inlineStr">
         <is>
@@ -31947,16 +31945,18 @@
         </is>
       </c>
       <c r="J26" s="24" t="n">
-        <v>0.7342596256130441</v>
+        <v>0.7298353476776207</v>
       </c>
       <c r="K26" s="24" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="L26" s="24" t="n">
-        <v>0.98458296</v>
+        <v>0.792</v>
+      </c>
+      <c r="L26" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="M26" s="24" t="n">
-        <v>6.581567</v>
+        <v>0.10938541</v>
       </c>
     </row>
     <row r="27" ht="17" customHeight="1">
@@ -31965,22 +31965,22 @@
       </c>
       <c r="C27" s="26" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>FNC.V</t>
         </is>
       </c>
       <c r="D27" s="18" t="inlineStr">
         <is>
-          <t>Katapult Holdings Inc. Common Stock</t>
+          <t>Fancamp Exploration Ltd.</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="G27" s="21" t="inlineStr">
@@ -31989,26 +31989,26 @@
         </is>
       </c>
       <c r="H27" s="22" t="n">
-        <v>32688298</v>
-      </c>
-      <c r="I27" s="25" t="inlineStr">
-        <is>
-          <t>UNRESEARCHED</t>
+        <v>25843393.62515116</v>
+      </c>
+      <c r="I27" s="23" t="inlineStr">
+        <is>
+          <t>GREEN</t>
         </is>
       </c>
       <c r="J27" s="24" t="n">
-        <v>0.7298353476776207</v>
+        <v>0.7274859584857709</v>
       </c>
       <c r="K27" s="24" t="n">
-        <v>0.792</v>
-      </c>
-      <c r="L27" s="27" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="L27" s="24" t="n">
+        <v>0.62500006</v>
+      </c>
+      <c r="M27" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
-      </c>
-      <c r="M27" s="24" t="n">
-        <v>0.10938541</v>
       </c>
     </row>
     <row r="28" ht="17" customHeight="1">
@@ -32017,50 +32017,48 @@
       </c>
       <c r="C28" s="26" t="inlineStr">
         <is>
-          <t>FNC.V</t>
+          <t>OPBK</t>
         </is>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Fancamp Exploration Ltd.</t>
+          <t>OP Bancorp</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>25843393.62515116</v>
-      </c>
-      <c r="I28" s="23" t="inlineStr">
-        <is>
-          <t>GREEN</t>
+        <v>229222336</v>
+      </c>
+      <c r="I28" s="25" t="inlineStr">
+        <is>
+          <t>UNRESEARCHED</t>
         </is>
       </c>
       <c r="J28" s="24" t="n">
-        <v>0.7274859584857709</v>
+        <v>0.7274389476177404</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L28" s="24" t="n">
-        <v>0.62500006</v>
-      </c>
-      <c r="M28" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.9850231</v>
+      </c>
+      <c r="M28" s="24" t="n">
+        <v>2.4451687</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-render all books after container restart on fully-corrected data
All render-managed books regenerated on the archetype-review-corrected
data (136 archetypes incl. the 2 revived dead gates and the currency/
normalization fixes). 180 checks 0 FAIL 0 WARN, mutation 32/0,
conformance 15/15.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -31795,12 +31795,12 @@
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SBCWW</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>Sbc Medical Group Holdings Incorporated</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
@@ -31810,7 +31810,7 @@
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
@@ -31819,7 +31819,7 @@
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>12773946</v>
+        <v>31542409.9725</v>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
@@ -31827,23 +31827,21 @@
         </is>
       </c>
       <c r="J12" s="24" t="n">
-        <v>0.8427237197322167</v>
+        <v>0.8417304836155266</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>0.571</v>
+        <v>0.8</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>0.6015113</v>
+        <v>0.12247278</v>
       </c>
       <c r="M12" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N12" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="N12" s="24" t="n">
+        <v>0.1781037290964673</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -31852,31 +31850,31 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>SBCWW</t>
+          <t>DC-A.TO</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Sbc Medical Group Holdings Incorporated</t>
+          <t>Dundee Corporation</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H13" s="22" t="n">
-        <v>31542409.9725</v>
+        <v>334198944.4364262</v>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
@@ -31884,13 +31882,13 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.8417304836155266</v>
+        <v>0.8416725320266993</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.8</v>
+        <v>0.891</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0.12247278</v>
+        <v>0.81739134</v>
       </c>
       <c r="M13" s="27" t="inlineStr">
         <is>
@@ -31898,7 +31896,7 @@
         </is>
       </c>
       <c r="N13" s="24" t="n">
-        <v>0.1781037290964673</v>
+        <v>46.262455</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -31907,31 +31905,31 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>DC-A.TO</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>Dundee Corporation</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H14" s="22" t="n">
-        <v>334198944.4364262</v>
+        <v>46763160</v>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
@@ -31939,13 +31937,13 @@
         </is>
       </c>
       <c r="J14" s="24" t="n">
-        <v>0.8416725320266993</v>
+        <v>0.8386666752381667</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>0.891</v>
+        <v>1</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0.81739134</v>
+        <v>0.69867694</v>
       </c>
       <c r="M14" s="27" t="inlineStr">
         <is>
@@ -31953,7 +31951,7 @@
         </is>
       </c>
       <c r="N14" s="24" t="n">
-        <v>46.262455</v>
+        <v>2.4335532</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -31962,12 +31960,12 @@
       </c>
       <c r="C15" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
@@ -31977,7 +31975,7 @@
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
@@ -31986,7 +31984,7 @@
         </is>
       </c>
       <c r="H15" s="22" t="n">
-        <v>46763160</v>
+        <v>12773946</v>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
@@ -31994,21 +31992,23 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.8386666752381667</v>
+        <v>0.832868113719865</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.69867694</v>
+        <v>0.6015113</v>
       </c>
       <c r="M15" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N15" s="24" t="n">
-        <v>2.4335532</v>
+      <c r="N15" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -32214,10 +32214,10 @@
         </is>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.8068228581375196</v>
+        <v>0.8035042382866744</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.828</v>
+        <v>0.803</v>
       </c>
       <c r="L19" s="24" t="n">
         <v>0.2269332554781938</v>
@@ -50742,10 +50742,10 @@
         </is>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.7483747819327972</v>
+        <v>0.7397178222661022</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>0.667</v>
+        <v>0.6</v>
       </c>
       <c r="L8" s="27" t="inlineStr">
         <is>
@@ -63517,10 +63517,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.6994979809618332</v>
+        <v>0.6964958437044864</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.825</v>
+        <v>0.8</v>
       </c>
       <c r="L9" s="24" t="n">
         <v>0.9437919</v>
@@ -63733,10 +63733,10 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.6496446992604653</v>
+        <v>0.6454348598041391</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.739</v>
+        <v>0.701</v>
       </c>
       <c r="L13" s="24" t="n">
         <v>0.33102494</v>
@@ -63945,10 +63945,10 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.6088780483119204</v>
+        <v>0.6047375032446598</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.588</v>
+        <v>0.55</v>
       </c>
       <c r="L17" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild all books with broadened post-reorg cohort
Regenerated the render-managed workbooks so the expanded post-reorg archetype
(1 -> 8 firers: GPOR, EXE, CHRD, WFRD, NE, VTOL, AMPY, DBD) surfaces across the
archetype, country, segment, and top-N books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -31722,12 +31722,12 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>TTEC</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>Ttec Holdings, Inc.</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -31737,16 +31737,16 @@
       </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H11" s="22" t="n">
-        <v>12457237</v>
+        <v>63345280</v>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
@@ -31754,23 +31754,19 @@
         </is>
       </c>
       <c r="J11" s="24" t="n">
-        <v>0.8444224464948391</v>
+        <v>0.8425192587847309</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.571</v>
+        <v>0.8</v>
       </c>
       <c r="L11" s="24" t="n">
-        <v>0.58659774</v>
-      </c>
-      <c r="M11" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N11" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.65628195</v>
+      </c>
+      <c r="M11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="24" t="n">
+        <v>0.031039892</v>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
@@ -31779,12 +31775,12 @@
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>TTEC</t>
+          <t>SBCWW</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Ttec Holdings, Inc.</t>
+          <t>Sbc Medical Group Holdings Incorporated</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
@@ -31794,16 +31790,16 @@
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>63345280</v>
+        <v>31542409.9725</v>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
@@ -31811,19 +31807,21 @@
         </is>
       </c>
       <c r="J12" s="24" t="n">
-        <v>0.8425192587847309</v>
+        <v>0.8415046914231734</v>
       </c>
       <c r="K12" s="24" t="n">
         <v>0.8</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>0.65628195</v>
-      </c>
-      <c r="M12" s="25" t="n">
-        <v>0</v>
+        <v>0.12441679</v>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
       <c r="N12" s="24" t="n">
-        <v>0.031039892</v>
+        <v>0.1781037290964673</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -31832,31 +31830,31 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>SBCWW</t>
+          <t>DC-A.TO</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Sbc Medical Group Holdings Incorporated</t>
+          <t>Dundee Corporation</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H13" s="22" t="n">
-        <v>31542409.9725</v>
+        <v>338077473.7864094</v>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
@@ -31864,13 +31862,13 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.8415046914231734</v>
+        <v>0.8403952351617557</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.8</v>
+        <v>0.891</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0.12441679</v>
+        <v>0.8268775</v>
       </c>
       <c r="M13" s="27" t="inlineStr">
         <is>
@@ -31878,7 +31876,7 @@
         </is>
       </c>
       <c r="N13" s="24" t="n">
-        <v>0.1781037290964673</v>
+        <v>46.79935</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -31887,31 +31885,31 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>DC-A.TO</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>Dundee Corporation</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H14" s="22" t="n">
-        <v>338077473.7864094</v>
+        <v>48653588</v>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
@@ -31919,13 +31917,13 @@
         </is>
       </c>
       <c r="J14" s="24" t="n">
-        <v>0.8403952351617557</v>
+        <v>0.8386666752381667</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>0.891</v>
+        <v>1</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0.8268775</v>
+        <v>0.7269213</v>
       </c>
       <c r="M14" s="27" t="inlineStr">
         <is>
@@ -31933,7 +31931,7 @@
         </is>
       </c>
       <c r="N14" s="24" t="n">
-        <v>46.79935</v>
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -31942,12 +31940,12 @@
       </c>
       <c r="C15" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
@@ -31957,7 +31955,7 @@
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
@@ -31966,7 +31964,7 @@
         </is>
       </c>
       <c r="H15" s="22" t="n">
-        <v>48653588</v>
+        <v>12457237</v>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
@@ -31974,21 +31972,23 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.8386666752381667</v>
+        <v>0.8345469739695329</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.58659774</v>
       </c>
       <c r="M15" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N15" s="24" t="n">
-        <v>2.5319312</v>
+      <c r="N15" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -32107,12 +32107,12 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>XNET</t>
+          <t>SSBI</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>Xunlei Ltd</t>
+          <t>Summit State Bank</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -32122,16 +32122,16 @@
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>318702240</v>
+        <v>85936024</v>
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
@@ -32139,13 +32139,13 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.8062111750244484</v>
+        <v>0.8033481199327791</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.828</v>
+        <v>0.95</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.2320380985386871</v>
+        <v>0.84785366</v>
       </c>
       <c r="M18" s="27" t="inlineStr">
         <is>
@@ -32153,7 +32153,7 @@
         </is>
       </c>
       <c r="N18" s="24" t="n">
-        <v>0.64597005</v>
+        <v>2.366666409627936</v>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
@@ -32162,12 +32162,12 @@
       </c>
       <c r="C19" s="28" t="inlineStr">
         <is>
-          <t>SSBI</t>
+          <t>XNET</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Summit State Bank</t>
+          <t>Xunlei Ltd</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -32177,16 +32177,16 @@
       </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="G19" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>85936024</v>
+        <v>318702240</v>
       </c>
       <c r="I19" s="26" t="inlineStr">
         <is>
@@ -32194,13 +32194,13 @@
         </is>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.8033481199327791</v>
+        <v>0.802895071145605</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.95</v>
+        <v>0.803</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>0.84785366</v>
+        <v>0.2320380985386871</v>
       </c>
       <c r="M19" s="27" t="inlineStr">
         <is>
@@ -32208,7 +32208,7 @@
         </is>
       </c>
       <c r="N19" s="24" t="n">
-        <v>2.366666409627936</v>
+        <v>0.64597005</v>
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
@@ -50718,10 +50718,10 @@
         </is>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.7483747819327972</v>
+        <v>0.7397178222661022</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>0.667</v>
+        <v>0.6</v>
       </c>
       <c r="L8" s="27" t="inlineStr">
         <is>
@@ -63491,10 +63491,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.6994979809618332</v>
+        <v>0.6964958437044864</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.825</v>
+        <v>0.8</v>
       </c>
       <c r="L9" s="24" t="n">
         <v>0.9437919</v>
@@ -63707,10 +63707,10 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.6496446992604653</v>
+        <v>0.6454348598041391</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.739</v>
+        <v>0.701</v>
       </c>
       <c r="L13" s="24" t="n">
         <v>0.33102494</v>
@@ -63919,10 +63919,10 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.6088780483119204</v>
+        <v>0.6047375032446598</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.588</v>
+        <v>0.55</v>
       </c>
       <c r="L17" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild all books after surgical audit batch 5
Regenerated the render-managed workbooks on the audited archetype set: the
conservative archetype_count collapse (3 same-thesis clusters), impairment-
robust spin viability, the recovered non-US OTC compounders (Nongfu/Anta/
Paycom), and the SOLS materials-spin sector correction are all reflected.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -31722,12 +31722,12 @@
       </c>
       <c r="C11" s="28" t="inlineStr">
         <is>
-          <t>TTEC</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D11" s="18" t="inlineStr">
         <is>
-          <t>Ttec Holdings, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -31737,16 +31737,16 @@
       </c>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H11" s="22" t="n">
-        <v>63345280</v>
+        <v>12457237</v>
       </c>
       <c r="I11" s="26" t="inlineStr">
         <is>
@@ -31754,19 +31754,23 @@
         </is>
       </c>
       <c r="J11" s="24" t="n">
-        <v>0.8425192587847309</v>
+        <v>0.8444224464948391</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.8</v>
+        <v>0.571</v>
       </c>
       <c r="L11" s="24" t="n">
-        <v>0.65628195</v>
-      </c>
-      <c r="M11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="24" t="n">
-        <v>0.031039892</v>
+        <v>0.58659774</v>
+      </c>
+      <c r="M11" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N11" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="17" customHeight="1">
@@ -31775,12 +31779,12 @@
       </c>
       <c r="C12" s="28" t="inlineStr">
         <is>
-          <t>SBCWW</t>
+          <t>TTEC</t>
         </is>
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>Sbc Medical Group Holdings Incorporated</t>
+          <t>Ttec Holdings, Inc.</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
@@ -31790,16 +31794,16 @@
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H12" s="22" t="n">
-        <v>31542409.9725</v>
+        <v>63345280</v>
       </c>
       <c r="I12" s="26" t="inlineStr">
         <is>
@@ -31807,21 +31811,19 @@
         </is>
       </c>
       <c r="J12" s="24" t="n">
-        <v>0.8415046914231734</v>
+        <v>0.8425192587847309</v>
       </c>
       <c r="K12" s="24" t="n">
         <v>0.8</v>
       </c>
       <c r="L12" s="24" t="n">
-        <v>0.12441679</v>
-      </c>
-      <c r="M12" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+        <v>0.65628195</v>
+      </c>
+      <c r="M12" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="N12" s="24" t="n">
-        <v>0.1781037290964673</v>
+        <v>0.031039892</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -31830,31 +31832,31 @@
       </c>
       <c r="C13" s="28" t="inlineStr">
         <is>
-          <t>DC-A.TO</t>
+          <t>SBCWW</t>
         </is>
       </c>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Dundee Corporation</t>
+          <t>Sbc Medical Group Holdings Incorporated</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>US</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>Consumer Staples</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H13" s="22" t="n">
-        <v>338077473.7864094</v>
+        <v>31542409.9725</v>
       </c>
       <c r="I13" s="26" t="inlineStr">
         <is>
@@ -31862,13 +31864,13 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.8403952351617557</v>
+        <v>0.8415046914231734</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.891</v>
+        <v>0.8</v>
       </c>
       <c r="L13" s="24" t="n">
-        <v>0.8268775</v>
+        <v>0.12441679</v>
       </c>
       <c r="M13" s="27" t="inlineStr">
         <is>
@@ -31876,7 +31878,7 @@
         </is>
       </c>
       <c r="N13" s="24" t="n">
-        <v>46.79935</v>
+        <v>0.1781037290964673</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -31885,31 +31887,31 @@
       </c>
       <c r="C14" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>DC-A.TO</t>
         </is>
       </c>
       <c r="D14" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Dundee Corporation</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CA</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H14" s="22" t="n">
-        <v>48653588</v>
+        <v>338077473.7864094</v>
       </c>
       <c r="I14" s="26" t="inlineStr">
         <is>
@@ -31917,13 +31919,13 @@
         </is>
       </c>
       <c r="J14" s="24" t="n">
-        <v>0.8386666752381667</v>
+        <v>0.8403952351617557</v>
       </c>
       <c r="K14" s="24" t="n">
-        <v>1</v>
+        <v>0.891</v>
       </c>
       <c r="L14" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.8268775</v>
       </c>
       <c r="M14" s="27" t="inlineStr">
         <is>
@@ -31931,7 +31933,7 @@
         </is>
       </c>
       <c r="N14" s="24" t="n">
-        <v>2.5319312</v>
+        <v>46.79935</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -31940,12 +31942,12 @@
       </c>
       <c r="C15" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D15" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
@@ -31955,7 +31957,7 @@
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G15" s="21" t="inlineStr">
@@ -31964,7 +31966,7 @@
         </is>
       </c>
       <c r="H15" s="22" t="n">
-        <v>12457237</v>
+        <v>48653588</v>
       </c>
       <c r="I15" s="26" t="inlineStr">
         <is>
@@ -31972,23 +31974,21 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.8345469739695329</v>
+        <v>0.8386666752381667</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L15" s="24" t="n">
-        <v>0.58659774</v>
+        <v>0.7269213</v>
       </c>
       <c r="M15" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N15" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="N15" s="24" t="n">
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="16" ht="17" customHeight="1">
@@ -32107,12 +32107,12 @@
       </c>
       <c r="C18" s="28" t="inlineStr">
         <is>
-          <t>SSBI</t>
+          <t>XNET</t>
         </is>
       </c>
       <c r="D18" s="18" t="inlineStr">
         <is>
-          <t>Summit State Bank</t>
+          <t>Xunlei Ltd</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -32122,16 +32122,16 @@
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="G18" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Small Cap</t>
         </is>
       </c>
       <c r="H18" s="22" t="n">
-        <v>85936024</v>
+        <v>318702240</v>
       </c>
       <c r="I18" s="26" t="inlineStr">
         <is>
@@ -32139,13 +32139,13 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.8033481199327791</v>
+        <v>0.8062111750244484</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.95</v>
+        <v>0.828</v>
       </c>
       <c r="L18" s="24" t="n">
-        <v>0.84785366</v>
+        <v>0.2320380985386871</v>
       </c>
       <c r="M18" s="27" t="inlineStr">
         <is>
@@ -32153,7 +32153,7 @@
         </is>
       </c>
       <c r="N18" s="24" t="n">
-        <v>2.366666409627936</v>
+        <v>0.64597005</v>
       </c>
     </row>
     <row r="19" ht="17" customHeight="1">
@@ -32162,12 +32162,12 @@
       </c>
       <c r="C19" s="28" t="inlineStr">
         <is>
-          <t>XNET</t>
+          <t>SSBI</t>
         </is>
       </c>
       <c r="D19" s="18" t="inlineStr">
         <is>
-          <t>Xunlei Ltd</t>
+          <t>Summit State Bank</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -32177,16 +32177,16 @@
       </c>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>Communication Services</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G19" s="21" t="inlineStr">
         <is>
-          <t>Small Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H19" s="22" t="n">
-        <v>318702240</v>
+        <v>85936024</v>
       </c>
       <c r="I19" s="26" t="inlineStr">
         <is>
@@ -32194,13 +32194,13 @@
         </is>
       </c>
       <c r="J19" s="24" t="n">
-        <v>0.802895071145605</v>
+        <v>0.8033481199327791</v>
       </c>
       <c r="K19" s="24" t="n">
-        <v>0.803</v>
+        <v>0.95</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>0.2320380985386871</v>
+        <v>0.84785366</v>
       </c>
       <c r="M19" s="27" t="inlineStr">
         <is>
@@ -32208,7 +32208,7 @@
         </is>
       </c>
       <c r="N19" s="24" t="n">
-        <v>0.64597005</v>
+        <v>2.366666409627936</v>
       </c>
     </row>
     <row r="20" ht="17" customHeight="1">
@@ -50718,10 +50718,10 @@
         </is>
       </c>
       <c r="J8" s="24" t="n">
-        <v>0.7397178222661022</v>
+        <v>0.7483747819327972</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="L8" s="27" t="inlineStr">
         <is>
@@ -63491,10 +63491,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.6964958437044864</v>
+        <v>0.6994979809618332</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="L9" s="24" t="n">
         <v>0.9437919</v>
@@ -63707,10 +63707,10 @@
         </is>
       </c>
       <c r="J13" s="24" t="n">
-        <v>0.6454348598041391</v>
+        <v>0.6496446992604653</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>0.701</v>
+        <v>0.739</v>
       </c>
       <c r="L13" s="24" t="n">
         <v>0.33102494</v>
@@ -63919,10 +63919,10 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.6047375032446598</v>
+        <v>0.6088780483119204</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.55</v>
+        <v>0.588</v>
       </c>
       <c r="L17" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild all books with arch_xr_contracted_backlog (RPO)
Regenerated the render-managed workbooks so the contracted-backlog XR archetype
(101 firers, RPO-based) surfaces across the archetype, country, segment and
top-N books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -12220,12 +12220,12 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>ANSGR.IS</t>
+          <t>MERIT.IS</t>
         </is>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Anadolu Anonim Turk Sigorta Sirketi</t>
+          <t>Merit Turizm Yatirim ve Isletme Anonim Sirketi</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
@@ -12235,16 +12235,16 @@
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>1153570162.652592</v>
+        <v>117290370.1971518</v>
       </c>
       <c r="I28" s="26" t="inlineStr">
         <is>
@@ -12252,19 +12252,19 @@
         </is>
       </c>
       <c r="J28" s="24" t="n">
-        <v>0.4875212062086694</v>
+        <v>0.4875787113980344</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>0.667</v>
+        <v>0.738</v>
       </c>
       <c r="L28" s="24" t="n">
-        <v>1.3284723</v>
+        <v>0.26461387</v>
       </c>
       <c r="M28" s="25" t="n">
-        <v>4.9000002</v>
+        <v>6.41</v>
       </c>
       <c r="N28" s="24" t="n">
-        <v>0.5073823</v>
+        <v>16.029314</v>
       </c>
     </row>
   </sheetData>
@@ -32007,12 +32007,12 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -32022,7 +32022,7 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
@@ -32031,7 +32031,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>48653588</v>
+        <v>12457237</v>
       </c>
       <c r="I16" s="26" t="inlineStr">
         <is>
@@ -32039,21 +32039,23 @@
         </is>
       </c>
       <c r="J16" s="24" t="n">
-        <v>0.8081594299047473</v>
+        <v>0.8164227183294704</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>1</v>
+        <v>0.571</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.58659774</v>
       </c>
       <c r="M16" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N16" s="24" t="n">
-        <v>2.5319312</v>
+      <c r="N16" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
@@ -32062,12 +32064,12 @@
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -32077,7 +32079,7 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
@@ -32086,7 +32088,7 @@
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>12457237</v>
+        <v>48653588</v>
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
@@ -32094,23 +32096,21 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.8068747010339026</v>
+        <v>0.8081594299047473</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>0.58659774</v>
+        <v>0.7269213</v>
       </c>
       <c r="M17" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N17" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="N17" s="24" t="n">
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
@@ -32151,10 +32151,10 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.802895071145605</v>
+        <v>0.8062111750244484</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.803</v>
+        <v>0.828</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>0.2320380985386871</v>
@@ -50737,10 +50737,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.7397178222661022</v>
+        <v>0.7483747819327972</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="L9" s="27" t="inlineStr">
         <is>
@@ -63573,10 +63573,10 @@
         </is>
       </c>
       <c r="J11" s="24" t="n">
-        <v>0.619711718787281</v>
+        <v>0.6223828899889503</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="L11" s="24" t="n">
         <v>0.9437919</v>
@@ -63789,10 +63789,10 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.5742798753931376</v>
+        <v>0.578025607501778</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.701</v>
+        <v>0.739</v>
       </c>
       <c r="L15" s="24" t="n">
         <v>0.33102494</v>
@@ -64058,10 +64058,10 @@
         </is>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.5520472864940897</v>
+        <v>0.555827069716932</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.55</v>
+        <v>0.588</v>
       </c>
       <c r="L20" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild all books with arch_xr_hidden_segment_compounder
Regenerated the render-managed workbooks (incl. the Forensic-XR book) so the new
hidden-segment-compounder archetype surfaces across the archetype, country,
segment, and top-N books.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -12220,12 +12220,12 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>MERIT.IS</t>
+          <t>ANSGR.IS</t>
         </is>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Merit Turizm Yatirim ve Isletme Anonim Sirketi</t>
+          <t>Anadolu Anonim Turk Sigorta Sirketi</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
@@ -12235,16 +12235,16 @@
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Financials</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Nano Cap</t>
+          <t>Micro Cap</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>117290370.1971518</v>
+        <v>1153570162.652592</v>
       </c>
       <c r="I28" s="26" t="inlineStr">
         <is>
@@ -12252,19 +12252,19 @@
         </is>
       </c>
       <c r="J28" s="24" t="n">
-        <v>0.4875787113980344</v>
+        <v>0.4875212062086694</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>0.738</v>
+        <v>0.667</v>
       </c>
       <c r="L28" s="24" t="n">
-        <v>0.26461387</v>
+        <v>1.3284723</v>
       </c>
       <c r="M28" s="25" t="n">
-        <v>6.41</v>
+        <v>4.9000002</v>
       </c>
       <c r="N28" s="24" t="n">
-        <v>16.029314</v>
+        <v>0.5073823</v>
       </c>
     </row>
   </sheetData>
@@ -32007,12 +32007,12 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -32022,7 +32022,7 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
@@ -32031,7 +32031,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>12457237</v>
+        <v>48653588</v>
       </c>
       <c r="I16" s="26" t="inlineStr">
         <is>
@@ -32039,23 +32039,21 @@
         </is>
       </c>
       <c r="J16" s="24" t="n">
-        <v>0.8164227183294704</v>
+        <v>0.8081594299047473</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>0.571</v>
+        <v>1</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>0.58659774</v>
+        <v>0.7269213</v>
       </c>
       <c r="M16" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N16" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="N16" s="24" t="n">
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
@@ -32064,12 +32062,12 @@
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -32079,7 +32077,7 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
@@ -32088,7 +32086,7 @@
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>48653588</v>
+        <v>12457237</v>
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
@@ -32096,21 +32094,23 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.8081594299047473</v>
+        <v>0.8068747010339026</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.58659774</v>
       </c>
       <c r="M17" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N17" s="24" t="n">
-        <v>2.5319312</v>
+      <c r="N17" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
@@ -32151,10 +32151,10 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.8062111750244484</v>
+        <v>0.802895071145605</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.828</v>
+        <v>0.803</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>0.2320380985386871</v>
@@ -50737,10 +50737,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.7483747819327972</v>
+        <v>0.7397178222661022</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.667</v>
+        <v>0.6</v>
       </c>
       <c r="L9" s="27" t="inlineStr">
         <is>
@@ -63573,10 +63573,10 @@
         </is>
       </c>
       <c r="J11" s="24" t="n">
-        <v>0.6223828899889503</v>
+        <v>0.619711718787281</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.825</v>
+        <v>0.8</v>
       </c>
       <c r="L11" s="24" t="n">
         <v>0.9437919</v>
@@ -63789,10 +63789,10 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.578025607501778</v>
+        <v>0.5742798753931376</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.739</v>
+        <v>0.701</v>
       </c>
       <c r="L15" s="24" t="n">
         <v>0.33102494</v>
@@ -64058,10 +64058,10 @@
         </is>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.555827069716932</v>
+        <v>0.5520472864940897</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.588</v>
+        <v>0.55</v>
       </c>
       <c r="L20" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>

<commit_message>
Rebuild full book set on Wave-2 + truly_xr data
Refresh the remaining non-legacy workbooks against the canonically-rebuilt
asymmetry_global / archetype_tags (Wave-2 forensic archetypes + truly_xr
composite): Harvard, NMS, NMS candidates, segment detail, country workbook,
country-archetype, country-inflection, OTC-archetype, FDB expansion. Combined
with the earlier archetype / forensic-XR / truly-XR rebuilds, this is the full
updated set.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pk8K7QpC1m36MYjRwkTznS
</commit_message>
<xml_diff>
--- a/asymmetry_nms_book.xlsx
+++ b/asymmetry_nms_book.xlsx
@@ -12220,12 +12220,12 @@
       </c>
       <c r="C28" s="28" t="inlineStr">
         <is>
-          <t>ANSGR.IS</t>
+          <t>MERIT.IS</t>
         </is>
       </c>
       <c r="D28" s="18" t="inlineStr">
         <is>
-          <t>Anadolu Anonim Turk Sigorta Sirketi</t>
+          <t>Merit Turizm Yatirim ve Isletme Anonim Sirketi</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
@@ -12235,16 +12235,16 @@
       </c>
       <c r="F28" s="20" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="G28" s="21" t="inlineStr">
         <is>
-          <t>Micro Cap</t>
+          <t>Nano Cap</t>
         </is>
       </c>
       <c r="H28" s="22" t="n">
-        <v>1153570162.652592</v>
+        <v>117290370.1971518</v>
       </c>
       <c r="I28" s="26" t="inlineStr">
         <is>
@@ -12252,19 +12252,19 @@
         </is>
       </c>
       <c r="J28" s="24" t="n">
-        <v>0.4875212062086694</v>
+        <v>0.4875787113980344</v>
       </c>
       <c r="K28" s="24" t="n">
-        <v>0.667</v>
+        <v>0.738</v>
       </c>
       <c r="L28" s="24" t="n">
-        <v>1.3284723</v>
+        <v>0.26461387</v>
       </c>
       <c r="M28" s="25" t="n">
-        <v>4.9000002</v>
+        <v>6.41</v>
       </c>
       <c r="N28" s="24" t="n">
-        <v>0.5073823</v>
+        <v>16.029314</v>
       </c>
     </row>
   </sheetData>
@@ -32007,12 +32007,12 @@
       </c>
       <c r="C16" s="28" t="inlineStr">
         <is>
-          <t>SCYX</t>
+          <t>BANL</t>
         </is>
       </c>
       <c r="D16" s="18" t="inlineStr">
         <is>
-          <t>SCYNEXIS, Inc.</t>
+          <t>Cbl International Limited</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
@@ -32022,7 +32022,7 @@
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>Health Care</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
@@ -32031,7 +32031,7 @@
         </is>
       </c>
       <c r="H16" s="22" t="n">
-        <v>48653588</v>
+        <v>12457237</v>
       </c>
       <c r="I16" s="26" t="inlineStr">
         <is>
@@ -32039,21 +32039,23 @@
         </is>
       </c>
       <c r="J16" s="24" t="n">
-        <v>0.8081594299047473</v>
+        <v>0.8164227183294704</v>
       </c>
       <c r="K16" s="24" t="n">
-        <v>1</v>
+        <v>0.571</v>
       </c>
       <c r="L16" s="24" t="n">
-        <v>0.7269213</v>
+        <v>0.58659774</v>
       </c>
       <c r="M16" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N16" s="24" t="n">
-        <v>2.5319312</v>
+      <c r="N16" s="27" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
       </c>
     </row>
     <row r="17" ht="17" customHeight="1">
@@ -32062,12 +32064,12 @@
       </c>
       <c r="C17" s="28" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>SCYX</t>
         </is>
       </c>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Cbl International Limited</t>
+          <t>SCYNEXIS, Inc.</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -32077,7 +32079,7 @@
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Health Care</t>
         </is>
       </c>
       <c r="G17" s="21" t="inlineStr">
@@ -32086,7 +32088,7 @@
         </is>
       </c>
       <c r="H17" s="22" t="n">
-        <v>12457237</v>
+        <v>48653588</v>
       </c>
       <c r="I17" s="26" t="inlineStr">
         <is>
@@ -32094,23 +32096,21 @@
         </is>
       </c>
       <c r="J17" s="24" t="n">
-        <v>0.8068747010339026</v>
+        <v>0.8081594299047473</v>
       </c>
       <c r="K17" s="24" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>0.58659774</v>
+        <v>0.7269213</v>
       </c>
       <c r="M17" s="27" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="N17" s="27" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
+      <c r="N17" s="24" t="n">
+        <v>2.5319312</v>
       </c>
     </row>
     <row r="18" ht="17" customHeight="1">
@@ -32151,10 +32151,10 @@
         </is>
       </c>
       <c r="J18" s="24" t="n">
-        <v>0.802895071145605</v>
+        <v>0.8062111750244484</v>
       </c>
       <c r="K18" s="24" t="n">
-        <v>0.803</v>
+        <v>0.828</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>0.2320380985386871</v>
@@ -50737,10 +50737,10 @@
         </is>
       </c>
       <c r="J9" s="24" t="n">
-        <v>0.7397178222661022</v>
+        <v>0.7483747819327972</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="L9" s="27" t="inlineStr">
         <is>
@@ -63573,10 +63573,10 @@
         </is>
       </c>
       <c r="J11" s="24" t="n">
-        <v>0.619711718787281</v>
+        <v>0.6223828899889503</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>0.8</v>
+        <v>0.825</v>
       </c>
       <c r="L11" s="24" t="n">
         <v>0.9437919</v>
@@ -63789,10 +63789,10 @@
         </is>
       </c>
       <c r="J15" s="24" t="n">
-        <v>0.5742798753931376</v>
+        <v>0.578025607501778</v>
       </c>
       <c r="K15" s="24" t="n">
-        <v>0.701</v>
+        <v>0.739</v>
       </c>
       <c r="L15" s="24" t="n">
         <v>0.33102494</v>
@@ -64058,10 +64058,10 @@
         </is>
       </c>
       <c r="J20" s="24" t="n">
-        <v>0.5520472864940897</v>
+        <v>0.555827069716932</v>
       </c>
       <c r="K20" s="24" t="n">
-        <v>0.55</v>
+        <v>0.588</v>
       </c>
       <c r="L20" s="24" t="n">
         <v>0.7176173</v>

</xml_diff>